<commit_message>
Rename actual Fast badge columns to actual O2D ≤ 5
Fast badge is stated O2D only. Label the o2d_actual_5 share as
actual O2D ≤ 5 in Excel headers, CSVs, and the control SQL alias.

Co-authored-by: et844p <et844p@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/weekend_shipping_pre_post/weekend_shipping_pre_post_supplier.xlsx
+++ b/output/weekend_shipping_pre_post/weekend_shipping_pre_post_supplier.xlsx
@@ -518,7 +518,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-31. Pre = 6 weeks before each warehouse’s first weekend-MSBD week. Post = enable week through 2026-08-16. Stated O2S = o2sumsbd (order date to supplier MSBD). Fast badge = stated O2D ≤ 5 days. Negative day deltas = faster.</t>
+          <t>Generated 2026-08-31. Pre = 6 weeks before each warehouse’s first weekend-MSBD week. Post = enable week through 2026-08-16. Stated O2S = o2sumsbd (order date to supplier MSBD). Fast badge = stated O2D ≤ 5 only (customer badge). Actual O2D ≤ 5 is delivery outcome, not a badge. Negative day deltas = faster.</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>o2d_stated_5</t>
+          <t>o2d_stated_5 — badge is stated only</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>o2d_actual_5</t>
+          <t>o2d_actual_5 — delivery outcome, not a badge</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>o2d_stated_5</t>
+          <t>o2d_stated_5 — badge is stated only</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>o2d_actual_5</t>
+          <t>o2d_actual_5 — delivery outcome, not a badge</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>o2d_stated_5</t>
+          <t>o2d_stated_5 — badge is stated only</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>o2d_actual_5</t>
+          <t>o2d_actual_5 — delivery outcome, not a badge</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>o2d_stated_5</t>
+          <t>o2d_stated_5 — badge is stated only</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>o2d_actual_5</t>
+          <t>o2d_actual_5 — delivery outcome, not a badge</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>o2d_stated_5</t>
+          <t>o2d_stated_5 — badge is stated only</t>
         </is>
       </c>
     </row>
@@ -1895,7 +1895,7 @@
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>o2d_actual_5</t>
+          <t>o2d_actual_5 — delivery outcome, not a badge</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2082,7 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>Negative stated O2S / O2D deltas mean the promise got faster. Positive badge deltas mean more 5-day (or 1-day O2S) orders.</t>
+          <t>Negative stated O2S / O2D deltas mean the promise got faster. Positive Fast badge deltas mean more stated-O2D≤5 orders.</t>
         </is>
       </c>
     </row>
@@ -2128,12 +2128,12 @@
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="23" customWidth="1" min="23" max="23"/>
-    <col width="24" customWidth="1" min="24" max="24"/>
-    <col width="25" customWidth="1" min="25" max="25"/>
+    <col width="33" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="21" max="21"/>
+    <col width="31" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="21" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
     <col width="16" customWidth="1" min="26" max="26"/>
     <col width="17" customWidth="1" min="27" max="27"/>
     <col width="18" customWidth="1" min="28" max="28"/>
@@ -2261,32 +2261,32 @@
       </c>
       <c r="T1" s="12" t="inlineStr">
         <is>
-          <t>pre_fast_badge</t>
+          <t>Pre Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="U1" s="12" t="inlineStr">
         <is>
-          <t>post_fast_badge</t>
+          <t>Post Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="V1" s="12" t="inlineStr">
         <is>
-          <t>delta_fast_badge</t>
+          <t>Δ Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="W1" s="12" t="inlineStr">
         <is>
-          <t>pre_actual_fast_badge</t>
+          <t>Pre actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="X1" s="12" t="inlineStr">
         <is>
-          <t>post_actual_fast_badge</t>
+          <t>Post actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="Y1" s="12" t="inlineStr">
         <is>
-          <t>delta_actual_fast_badge</t>
+          <t>Δ actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="Z1" s="12" t="inlineStr">
@@ -7808,165 +7808,165 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>28772</v>
+        <v>272293</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Linon CA 92408</t>
+          <t>AMEZIEL INC AW-TX 77489</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Linon</t>
+          <t>AMEZIEL INC</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Casegoods</t>
+          <t>APS AEOF</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Connor Henderson</t>
+          <t>Carl Li</t>
         </is>
       </c>
       <c r="G34" s="13" t="n">
         <v>46236</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>561</v>
+        <v>480</v>
       </c>
       <c r="I34" s="6" t="n">
         <v>178</v>
       </c>
       <c r="J34" s="6" t="n">
-        <v>-383</v>
+        <v>-302</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>3.092691622103387</v>
+        <v>2.479166666666667</v>
       </c>
       <c r="L34" s="7" t="n">
-        <v>1.421348314606742</v>
+        <v>1.455056179775281</v>
       </c>
       <c r="M34" s="8" t="n">
-        <v>-1.671343307496645</v>
+        <v>-1.024110486891386</v>
       </c>
       <c r="N34" s="10" t="n">
         <v>0</v>
       </c>
       <c r="O34" s="10" t="n">
-        <v>0.5617977528089888</v>
+        <v>0.5449438202247191</v>
       </c>
       <c r="P34" s="11" t="n">
-        <v>0.5617977528089888</v>
+        <v>0.5449438202247191</v>
       </c>
       <c r="Q34" s="7" t="n">
-        <v>5.768248175182482</v>
+        <v>4.442348008385745</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>5.844827586206897</v>
+        <v>4.232954545454546</v>
       </c>
       <c r="S34" s="8" t="n">
-        <v>0.07657941102441512</v>
+        <v>-0.2093934629311986</v>
       </c>
       <c r="T34" s="10" t="n">
-        <v>0.5935828877005348</v>
+        <v>0.8708333333333333</v>
       </c>
       <c r="U34" s="10" t="n">
-        <v>0.6685393258426966</v>
+        <v>0.9550561797752809</v>
       </c>
       <c r="V34" s="11" t="n">
-        <v>0.0749564381421618</v>
+        <v>0.08422284644194755</v>
       </c>
       <c r="W34" s="10" t="n">
-        <v>0.6167557932263814</v>
+        <v>0.8770833333333333</v>
       </c>
       <c r="X34" s="10" t="n">
-        <v>0.6404494382022472</v>
+        <v>0.8707865168539326</v>
       </c>
       <c r="Y34" s="11" t="n">
-        <v>0.02369364497586579</v>
+        <v>-0.006296816479400724</v>
       </c>
       <c r="Z34" s="7" t="n">
-        <v>1.339285714285714</v>
+        <v>1.579166666666667</v>
       </c>
       <c r="AA34" s="7" t="n">
-        <v>1.078651685393258</v>
+        <v>1.584269662921348</v>
       </c>
       <c r="AB34" s="8" t="n">
-        <v>-0.2606340288924558</v>
+        <v>0.005102996254681802</v>
       </c>
       <c r="AC34" s="7" t="n">
-        <v>5.083928571428571</v>
+        <v>4.222916666666666</v>
       </c>
       <c r="AD34" s="7" t="n">
-        <v>4.601123595505618</v>
+        <v>4.163841807909605</v>
       </c>
       <c r="AE34" s="8" t="n">
-        <v>-0.4828049759229538</v>
+        <v>-0.05907485875706175</v>
       </c>
       <c r="AF34" s="10" t="n">
-        <v>0.9946524064171123</v>
+        <v>0.9895833333333334</v>
       </c>
       <c r="AG34" s="10" t="n">
-        <v>1</v>
+        <v>0.8595505617977528</v>
       </c>
       <c r="AH34" s="11" t="n">
-        <v>0.005347593582887722</v>
+        <v>-0.1300327715355806</v>
       </c>
       <c r="AI34" s="10" t="n">
-        <v>0.8228980322003577</v>
+        <v>0.9331941544885177</v>
       </c>
       <c r="AJ34" s="10" t="n">
-        <v>0.7752808988764045</v>
+        <v>0.847457627118644</v>
       </c>
       <c r="AK34" s="11" t="n">
-        <v>-0.04761713332395323</v>
+        <v>-0.08573652736987369</v>
       </c>
       <c r="AL34" s="6" t="n">
-        <v>3.000000000000012</v>
+        <v>4.999999999999982</v>
       </c>
       <c r="AM34" s="6" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="AN34" s="6" t="n">
-        <v>-3.000000000000012</v>
+        <v>20.00000000000002</v>
       </c>
       <c r="AO34" s="10" t="n">
-        <v>0.0035650623885918</v>
+        <v>0.002083333333333333</v>
       </c>
       <c r="AP34" s="10" t="n">
         <v>0.9719101123595506</v>
       </c>
       <c r="AQ34" s="11" t="n">
-        <v>0.9683450499709588</v>
+        <v>0.9698267790262173</v>
       </c>
       <c r="AR34" s="10" t="n">
-        <v>0.6702317290552585</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="AS34" s="10" t="n">
-        <v>0.8089887640449438</v>
+        <v>0.8426966292134831</v>
       </c>
       <c r="AT34" s="11" t="n">
-        <v>0.1387570349896853</v>
+        <v>-0.07397003745318353</v>
       </c>
       <c r="AU34" s="10" t="n">
-        <v>0.05</v>
+        <v>0.004166666666666667</v>
       </c>
       <c r="AV34" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AW34" s="11" t="n">
-        <v>-0.05</v>
+        <v>-0.004166666666666667</v>
       </c>
       <c r="AX34" s="10" t="n">
-        <v>0.6214285714285714</v>
+        <v>0.9125</v>
       </c>
       <c r="AY34" s="10" t="n">
-        <v>0.8089887640449438</v>
+        <v>0.8426966292134831</v>
       </c>
       <c r="AZ34" s="11" t="n">
-        <v>0.1875601926163724</v>
+        <v>-0.06980337078651688</v>
       </c>
     </row>
     <row r="35">
@@ -7976,165 +7976,165 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>272293</v>
+        <v>28772</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AMEZIEL INC AW-TX 77489</t>
+          <t>Linon CA 92408</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>AMEZIEL INC</t>
+          <t>Linon</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>APS AEOF</t>
+          <t>Casegoods</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Carl Li</t>
+          <t>Connor Henderson</t>
         </is>
       </c>
       <c r="G35" s="13" t="n">
         <v>46236</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>480</v>
+        <v>561</v>
       </c>
       <c r="I35" s="6" t="n">
         <v>178</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>-302</v>
+        <v>-383</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>2.479166666666667</v>
+        <v>3.092691622103387</v>
       </c>
       <c r="L35" s="7" t="n">
-        <v>1.455056179775281</v>
+        <v>1.421348314606742</v>
       </c>
       <c r="M35" s="8" t="n">
-        <v>-1.024110486891386</v>
+        <v>-1.671343307496645</v>
       </c>
       <c r="N35" s="10" t="n">
         <v>0</v>
       </c>
       <c r="O35" s="10" t="n">
-        <v>0.5449438202247191</v>
+        <v>0.5617977528089888</v>
       </c>
       <c r="P35" s="11" t="n">
-        <v>0.5449438202247191</v>
+        <v>0.5617977528089888</v>
       </c>
       <c r="Q35" s="7" t="n">
-        <v>4.442348008385745</v>
+        <v>5.768248175182482</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>4.232954545454546</v>
+        <v>5.844827586206897</v>
       </c>
       <c r="S35" s="8" t="n">
-        <v>-0.2093934629311986</v>
+        <v>0.07657941102441512</v>
       </c>
       <c r="T35" s="10" t="n">
-        <v>0.8708333333333333</v>
+        <v>0.5935828877005348</v>
       </c>
       <c r="U35" s="10" t="n">
-        <v>0.9550561797752809</v>
+        <v>0.6685393258426966</v>
       </c>
       <c r="V35" s="11" t="n">
-        <v>0.08422284644194755</v>
+        <v>0.0749564381421618</v>
       </c>
       <c r="W35" s="10" t="n">
-        <v>0.8770833333333333</v>
+        <v>0.6167557932263814</v>
       </c>
       <c r="X35" s="10" t="n">
-        <v>0.8707865168539326</v>
+        <v>0.6404494382022472</v>
       </c>
       <c r="Y35" s="11" t="n">
-        <v>-0.006296816479400724</v>
+        <v>0.02369364497586579</v>
       </c>
       <c r="Z35" s="7" t="n">
-        <v>1.579166666666667</v>
+        <v>1.339285714285714</v>
       </c>
       <c r="AA35" s="7" t="n">
-        <v>1.584269662921348</v>
+        <v>1.078651685393258</v>
       </c>
       <c r="AB35" s="8" t="n">
-        <v>0.005102996254681802</v>
+        <v>-0.2606340288924558</v>
       </c>
       <c r="AC35" s="7" t="n">
-        <v>4.222916666666666</v>
+        <v>5.083928571428571</v>
       </c>
       <c r="AD35" s="7" t="n">
-        <v>4.163841807909605</v>
+        <v>4.601123595505618</v>
       </c>
       <c r="AE35" s="8" t="n">
-        <v>-0.05907485875706175</v>
+        <v>-0.4828049759229538</v>
       </c>
       <c r="AF35" s="10" t="n">
-        <v>0.9895833333333334</v>
+        <v>0.9946524064171123</v>
       </c>
       <c r="AG35" s="10" t="n">
-        <v>0.8595505617977528</v>
+        <v>1</v>
       </c>
       <c r="AH35" s="11" t="n">
-        <v>-0.1300327715355806</v>
+        <v>0.005347593582887722</v>
       </c>
       <c r="AI35" s="10" t="n">
-        <v>0.9331941544885177</v>
+        <v>0.8228980322003577</v>
       </c>
       <c r="AJ35" s="10" t="n">
-        <v>0.847457627118644</v>
+        <v>0.7752808988764045</v>
       </c>
       <c r="AK35" s="11" t="n">
-        <v>-0.08573652736987369</v>
+        <v>-0.04761713332395323</v>
       </c>
       <c r="AL35" s="6" t="n">
-        <v>4.999999999999982</v>
+        <v>3.000000000000012</v>
       </c>
       <c r="AM35" s="6" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="AN35" s="6" t="n">
-        <v>20.00000000000002</v>
+        <v>-3.000000000000012</v>
       </c>
       <c r="AO35" s="10" t="n">
-        <v>0.002083333333333333</v>
+        <v>0.0035650623885918</v>
       </c>
       <c r="AP35" s="10" t="n">
         <v>0.9719101123595506</v>
       </c>
       <c r="AQ35" s="11" t="n">
-        <v>0.9698267790262173</v>
+        <v>0.9683450499709588</v>
       </c>
       <c r="AR35" s="10" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.6702317290552585</v>
       </c>
       <c r="AS35" s="10" t="n">
-        <v>0.8426966292134831</v>
+        <v>0.8089887640449438</v>
       </c>
       <c r="AT35" s="11" t="n">
-        <v>-0.07397003745318353</v>
+        <v>0.1387570349896853</v>
       </c>
       <c r="AU35" s="10" t="n">
-        <v>0.004166666666666667</v>
+        <v>0.05</v>
       </c>
       <c r="AV35" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AW35" s="11" t="n">
-        <v>-0.004166666666666667</v>
+        <v>-0.05</v>
       </c>
       <c r="AX35" s="10" t="n">
-        <v>0.9125</v>
+        <v>0.6214285714285714</v>
       </c>
       <c r="AY35" s="10" t="n">
-        <v>0.8426966292134831</v>
+        <v>0.8089887640449438</v>
       </c>
       <c r="AZ35" s="11" t="n">
-        <v>-0.06980337078651688</v>
+        <v>0.1875601926163724</v>
       </c>
     </row>
     <row r="36">
@@ -11336,21 +11336,21 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>327749</v>
+        <v>356699</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>无忧达美西区CAJW02</t>
+          <t>shanghaihuzidianzishangwuyouxiangongsi NJ 08016</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Hong Kong Baojia International Limited</t>
+          <t>Hong Kong HuaYa Trade Limited</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>APS</t>
+          <t>APS Home Improvement</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -11362,139 +11362,139 @@
         <v>46236</v>
       </c>
       <c r="H55" s="6" t="n">
-        <v>297</v>
+        <v>368</v>
       </c>
       <c r="I55" s="6" t="n">
         <v>114</v>
       </c>
       <c r="J55" s="6" t="n">
-        <v>-183</v>
+        <v>-254</v>
       </c>
       <c r="K55" s="7" t="n">
-        <v>2.602693602693603</v>
+        <v>2.323369565217391</v>
       </c>
       <c r="L55" s="7" t="n">
-        <v>1.535087719298246</v>
+        <v>1.210526315789474</v>
       </c>
       <c r="M55" s="8" t="n">
-        <v>-1.067605883395357</v>
+        <v>-1.112843249427917</v>
       </c>
       <c r="N55" s="10" t="n">
         <v>0</v>
       </c>
       <c r="O55" s="10" t="n">
-        <v>0.4736842105263158</v>
+        <v>0.5614035087719298</v>
       </c>
       <c r="P55" s="11" t="n">
-        <v>0.4736842105263158</v>
+        <v>0.5614035087719298</v>
       </c>
       <c r="Q55" s="7" t="n">
-        <v>5.833910034602076</v>
+        <v>4.544198895027624</v>
       </c>
       <c r="R55" s="7" t="n">
-        <v>5.245454545454545</v>
+        <v>4.178571428571429</v>
       </c>
       <c r="S55" s="8" t="n">
-        <v>-0.5884554891475311</v>
+        <v>-0.3656274664561954</v>
       </c>
       <c r="T55" s="10" t="n">
-        <v>0.5387205387205387</v>
+        <v>0.8858695652173914</v>
       </c>
       <c r="U55" s="10" t="n">
-        <v>0.6578947368421053</v>
+        <v>0.9385964912280702</v>
       </c>
       <c r="V55" s="11" t="n">
-        <v>0.1191741981215666</v>
+        <v>0.05272692601067885</v>
       </c>
       <c r="W55" s="10" t="n">
-        <v>0.5858585858585859</v>
+        <v>0.9375</v>
       </c>
       <c r="X55" s="10" t="n">
-        <v>0.5350877192982456</v>
+        <v>0.9649122807017544</v>
       </c>
       <c r="Y55" s="11" t="n">
-        <v>-0.05077086656034024</v>
+        <v>0.02741228070175439</v>
       </c>
       <c r="Z55" s="7" t="n">
-        <v>1.872053872053872</v>
+        <v>0.7880434782608695</v>
       </c>
       <c r="AA55" s="7" t="n">
-        <v>1.719298245614035</v>
+        <v>0.6140350877192983</v>
       </c>
       <c r="AB55" s="8" t="n">
-        <v>-0.1527556264398369</v>
+        <v>-0.1740083905415712</v>
       </c>
       <c r="AC55" s="7" t="n">
-        <v>5.700336700336701</v>
+        <v>3.551630434782609</v>
       </c>
       <c r="AD55" s="7" t="n">
-        <v>5.309734513274337</v>
+        <v>3.473684210526316</v>
       </c>
       <c r="AE55" s="8" t="n">
-        <v>-0.3906021870623642</v>
+        <v>-0.07794622425629294</v>
       </c>
       <c r="AF55" s="10" t="n">
-        <v>0.9898989898989899</v>
+        <v>0.9972826086956522</v>
       </c>
       <c r="AG55" s="10" t="n">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="AH55" s="11" t="n">
-        <v>-0.1565656565656566</v>
+        <v>0.002717391304347783</v>
       </c>
       <c r="AI55" s="10" t="n">
-        <v>0.9054054054054054</v>
+        <v>0.9482288828337875</v>
       </c>
       <c r="AJ55" s="10" t="n">
-        <v>0.6991150442477876</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="AK55" s="11" t="n">
-        <v>-0.2062903611576178</v>
+        <v>-0.05349204072852431</v>
       </c>
       <c r="AL55" s="6" t="n">
-        <v>2.999999999999986</v>
+        <v>0.999999999999984</v>
       </c>
       <c r="AM55" s="6" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="AN55" s="6" t="n">
-        <v>16.00000000000001</v>
+        <v>-0.999999999999984</v>
       </c>
       <c r="AO55" s="10" t="n">
-        <v>0.003367003367003367</v>
+        <v>0.002717391304347826</v>
       </c>
       <c r="AP55" s="10" t="n">
-        <v>0.9912280701754386</v>
+        <v>0.8859649122807017</v>
       </c>
       <c r="AQ55" s="11" t="n">
-        <v>0.9878610668084352</v>
+        <v>0.883247520976354</v>
       </c>
       <c r="AR55" s="10" t="n">
-        <v>0.7138047138047138</v>
+        <v>0.7608695652173914</v>
       </c>
       <c r="AS55" s="10" t="n">
-        <v>0.8245614035087719</v>
+        <v>0.8070175438596491</v>
       </c>
       <c r="AT55" s="11" t="n">
-        <v>0.1107566897040582</v>
+        <v>0.04614797864225773</v>
       </c>
       <c r="AU55" s="10" t="n">
-        <v>0</v>
+        <v>0.3315217391304348</v>
       </c>
       <c r="AV55" s="10" t="n">
-        <v>0</v>
+        <v>0.4385964912280702</v>
       </c>
       <c r="AW55" s="11" t="n">
-        <v>0</v>
+        <v>0.1070747520976354</v>
       </c>
       <c r="AX55" s="10" t="n">
-        <v>0.7138047138047138</v>
+        <v>0.4293478260869565</v>
       </c>
       <c r="AY55" s="10" t="n">
-        <v>0.8245614035087719</v>
+        <v>0.3684210526315789</v>
       </c>
       <c r="AZ55" s="11" t="n">
-        <v>0.1107566897040582</v>
+        <v>-0.06092677345537761</v>
       </c>
     </row>
     <row r="56">
@@ -11504,21 +11504,21 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>356699</v>
+        <v>327749</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>shanghaihuzidianzishangwuyouxiangongsi NJ 08016</t>
+          <t>无忧达美西区CAJW02</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Hong Kong HuaYa Trade Limited</t>
+          <t>Hong Kong Baojia International Limited</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>APS Home Improvement</t>
+          <t>APS</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -11530,139 +11530,139 @@
         <v>46236</v>
       </c>
       <c r="H56" s="6" t="n">
-        <v>368</v>
+        <v>297</v>
       </c>
       <c r="I56" s="6" t="n">
         <v>114</v>
       </c>
       <c r="J56" s="6" t="n">
-        <v>-254</v>
+        <v>-183</v>
       </c>
       <c r="K56" s="7" t="n">
-        <v>2.323369565217391</v>
+        <v>2.602693602693603</v>
       </c>
       <c r="L56" s="7" t="n">
-        <v>1.210526315789474</v>
+        <v>1.535087719298246</v>
       </c>
       <c r="M56" s="8" t="n">
-        <v>-1.112843249427917</v>
+        <v>-1.067605883395357</v>
       </c>
       <c r="N56" s="10" t="n">
         <v>0</v>
       </c>
       <c r="O56" s="10" t="n">
-        <v>0.5614035087719298</v>
+        <v>0.4736842105263158</v>
       </c>
       <c r="P56" s="11" t="n">
-        <v>0.5614035087719298</v>
+        <v>0.4736842105263158</v>
       </c>
       <c r="Q56" s="7" t="n">
-        <v>4.544198895027624</v>
+        <v>5.833910034602076</v>
       </c>
       <c r="R56" s="7" t="n">
-        <v>4.178571428571429</v>
+        <v>5.245454545454545</v>
       </c>
       <c r="S56" s="8" t="n">
-        <v>-0.3656274664561954</v>
+        <v>-0.5884554891475311</v>
       </c>
       <c r="T56" s="10" t="n">
-        <v>0.8858695652173914</v>
+        <v>0.5387205387205387</v>
       </c>
       <c r="U56" s="10" t="n">
-        <v>0.9385964912280702</v>
+        <v>0.6578947368421053</v>
       </c>
       <c r="V56" s="11" t="n">
-        <v>0.05272692601067885</v>
+        <v>0.1191741981215666</v>
       </c>
       <c r="W56" s="10" t="n">
-        <v>0.9375</v>
+        <v>0.5858585858585859</v>
       </c>
       <c r="X56" s="10" t="n">
-        <v>0.9649122807017544</v>
+        <v>0.5350877192982456</v>
       </c>
       <c r="Y56" s="11" t="n">
-        <v>0.02741228070175439</v>
+        <v>-0.05077086656034024</v>
       </c>
       <c r="Z56" s="7" t="n">
-        <v>0.7880434782608695</v>
+        <v>1.872053872053872</v>
       </c>
       <c r="AA56" s="7" t="n">
-        <v>0.6140350877192983</v>
+        <v>1.719298245614035</v>
       </c>
       <c r="AB56" s="8" t="n">
-        <v>-0.1740083905415712</v>
+        <v>-0.1527556264398369</v>
       </c>
       <c r="AC56" s="7" t="n">
-        <v>3.551630434782609</v>
+        <v>5.700336700336701</v>
       </c>
       <c r="AD56" s="7" t="n">
-        <v>3.473684210526316</v>
+        <v>5.309734513274337</v>
       </c>
       <c r="AE56" s="8" t="n">
-        <v>-0.07794622425629294</v>
+        <v>-0.3906021870623642</v>
       </c>
       <c r="AF56" s="10" t="n">
-        <v>0.9972826086956522</v>
+        <v>0.9898989898989899</v>
       </c>
       <c r="AG56" s="10" t="n">
-        <v>1</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="AH56" s="11" t="n">
-        <v>0.002717391304347783</v>
+        <v>-0.1565656565656566</v>
       </c>
       <c r="AI56" s="10" t="n">
-        <v>0.9482288828337875</v>
+        <v>0.9054054054054054</v>
       </c>
       <c r="AJ56" s="10" t="n">
-        <v>0.8947368421052632</v>
+        <v>0.6991150442477876</v>
       </c>
       <c r="AK56" s="11" t="n">
-        <v>-0.05349204072852431</v>
+        <v>-0.2062903611576178</v>
       </c>
       <c r="AL56" s="6" t="n">
-        <v>0.999999999999984</v>
+        <v>2.999999999999986</v>
       </c>
       <c r="AM56" s="6" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="AN56" s="6" t="n">
-        <v>-0.999999999999984</v>
+        <v>16.00000000000001</v>
       </c>
       <c r="AO56" s="10" t="n">
-        <v>0.002717391304347826</v>
+        <v>0.003367003367003367</v>
       </c>
       <c r="AP56" s="10" t="n">
-        <v>0.8859649122807017</v>
+        <v>0.9912280701754386</v>
       </c>
       <c r="AQ56" s="11" t="n">
-        <v>0.883247520976354</v>
+        <v>0.9878610668084352</v>
       </c>
       <c r="AR56" s="10" t="n">
-        <v>0.7608695652173914</v>
+        <v>0.7138047138047138</v>
       </c>
       <c r="AS56" s="10" t="n">
-        <v>0.8070175438596491</v>
+        <v>0.8245614035087719</v>
       </c>
       <c r="AT56" s="11" t="n">
-        <v>0.04614797864225773</v>
+        <v>0.1107566897040582</v>
       </c>
       <c r="AU56" s="10" t="n">
-        <v>0.3315217391304348</v>
+        <v>0</v>
       </c>
       <c r="AV56" s="10" t="n">
-        <v>0.4385964912280702</v>
+        <v>0</v>
       </c>
       <c r="AW56" s="11" t="n">
-        <v>0.1070747520976354</v>
+        <v>0</v>
       </c>
       <c r="AX56" s="10" t="n">
-        <v>0.4293478260869565</v>
+        <v>0.7138047138047138</v>
       </c>
       <c r="AY56" s="10" t="n">
-        <v>0.3684210526315789</v>
+        <v>0.8245614035087719</v>
       </c>
       <c r="AZ56" s="11" t="n">
-        <v>-0.06092677345537761</v>
+        <v>0.1107566897040582</v>
       </c>
     </row>
     <row r="57">
@@ -11672,165 +11672,165 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>12397</v>
+        <v>370173</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Ashley Furniture WI 54612</t>
+          <t>aifei(shanghai)kejiyouxiangongsi GA 30517</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Ashley Furniture</t>
+          <t>aifei(shanghai)kejiyouxiangongsi</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Upholstery</t>
+          <t>APS K&amp;D</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Anne Marie Conde</t>
+          <t>Eve Deng</t>
         </is>
       </c>
       <c r="G57" s="13" t="n">
         <v>46236</v>
       </c>
       <c r="H57" s="6" t="n">
-        <v>310</v>
+        <v>190</v>
       </c>
       <c r="I57" s="6" t="n">
         <v>113</v>
       </c>
       <c r="J57" s="6" t="n">
-        <v>-197</v>
+        <v>-77</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>1.935483870967742</v>
+        <v>2.552631578947369</v>
       </c>
       <c r="L57" s="7" t="n">
-        <v>1.265486725663717</v>
+        <v>1.849557522123894</v>
       </c>
       <c r="M57" s="8" t="n">
-        <v>-0.6699971453040252</v>
+        <v>-0.7030740568234748</v>
       </c>
       <c r="N57" s="10" t="n">
         <v>0</v>
       </c>
       <c r="O57" s="10" t="n">
+        <v>0.3628318584070797</v>
+      </c>
+      <c r="P57" s="11" t="n">
+        <v>0.3628318584070797</v>
+      </c>
+      <c r="Q57" s="7" t="n">
+        <v>4.579787234042553</v>
+      </c>
+      <c r="R57" s="7" t="n">
+        <v>4.433628318584071</v>
+      </c>
+      <c r="S57" s="8" t="n">
+        <v>-0.1461589154584821</v>
+      </c>
+      <c r="T57" s="10" t="n">
+        <v>0.9368421052631579</v>
+      </c>
+      <c r="U57" s="10" t="n">
+        <v>0.9823008849557522</v>
+      </c>
+      <c r="V57" s="11" t="n">
+        <v>0.04545877969259426</v>
+      </c>
+      <c r="W57" s="10" t="n">
+        <v>0.9105263157894737</v>
+      </c>
+      <c r="X57" s="10" t="n">
+        <v>0.9557522123893806</v>
+      </c>
+      <c r="Y57" s="11" t="n">
+        <v>0.04522589659990683</v>
+      </c>
+      <c r="Z57" s="7" t="n">
+        <v>1.768421052631579</v>
+      </c>
+      <c r="AA57" s="7" t="n">
+        <v>1.778761061946903</v>
+      </c>
+      <c r="AB57" s="8" t="n">
+        <v>0.01034000931532386</v>
+      </c>
+      <c r="AC57" s="7" t="n">
+        <v>4.347368421052631</v>
+      </c>
+      <c r="AD57" s="7" t="n">
+        <v>4.141592920353983</v>
+      </c>
+      <c r="AE57" s="8" t="n">
+        <v>-0.2057755006986488</v>
+      </c>
+      <c r="AF57" s="10" t="n">
+        <v>0.9842105263157894</v>
+      </c>
+      <c r="AG57" s="10" t="n">
+        <v>0.5929203539823009</v>
+      </c>
+      <c r="AH57" s="11" t="n">
+        <v>-0.3912901723334885</v>
+      </c>
+      <c r="AI57" s="10" t="n">
+        <v>0.8631578947368421</v>
+      </c>
+      <c r="AJ57" s="10" t="n">
+        <v>0.9292035398230089</v>
+      </c>
+      <c r="AK57" s="11" t="n">
+        <v>0.06604564508616673</v>
+      </c>
+      <c r="AL57" s="6" t="n">
+        <v>3.000000000000009</v>
+      </c>
+      <c r="AM57" s="6" t="n">
+        <v>45.99999999999999</v>
+      </c>
+      <c r="AN57" s="6" t="n">
+        <v>42.99999999999999</v>
+      </c>
+      <c r="AO57" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP57" s="10" t="n">
+        <v>0.5575221238938053</v>
+      </c>
+      <c r="AQ57" s="11" t="n">
+        <v>0.5575221238938053</v>
+      </c>
+      <c r="AR57" s="10" t="n">
+        <v>0.7789473684210526</v>
+      </c>
+      <c r="AS57" s="10" t="n">
+        <v>0.5663716814159292</v>
+      </c>
+      <c r="AT57" s="11" t="n">
+        <v>-0.2125756870051234</v>
+      </c>
+      <c r="AU57" s="10" t="n">
+        <v>0.01052631578947368</v>
+      </c>
+      <c r="AV57" s="10" t="n">
+        <v>0.06194690265486726</v>
+      </c>
+      <c r="AW57" s="11" t="n">
+        <v>0.05142058686539357</v>
+      </c>
+      <c r="AX57" s="10" t="n">
+        <v>0.7684210526315789</v>
+      </c>
+      <c r="AY57" s="10" t="n">
         <v>0.504424778761062</v>
       </c>
-      <c r="P57" s="11" t="n">
-        <v>0.504424778761062</v>
-      </c>
-      <c r="Q57" s="7" t="n">
-        <v>3.983221476510067</v>
-      </c>
-      <c r="R57" s="7" t="n">
-        <v>4.086538461538462</v>
-      </c>
-      <c r="S57" s="8" t="n">
-        <v>0.1033169850283944</v>
-      </c>
-      <c r="T57" s="10" t="n">
-        <v>0.8935483870967742</v>
-      </c>
-      <c r="U57" s="10" t="n">
-        <v>0.8584070796460177</v>
-      </c>
-      <c r="V57" s="11" t="n">
-        <v>-0.0351413074507565</v>
-      </c>
-      <c r="W57" s="10" t="n">
-        <v>0.8870967741935484</v>
-      </c>
-      <c r="X57" s="10" t="n">
-        <v>0.8849557522123894</v>
-      </c>
-      <c r="Y57" s="11" t="n">
-        <v>-0.002141021981158953</v>
-      </c>
-      <c r="Z57" s="7" t="n">
-        <v>0.6071428571428571</v>
-      </c>
-      <c r="AA57" s="7" t="n">
-        <v>0.5929203539823009</v>
-      </c>
-      <c r="AB57" s="8" t="n">
-        <v>-0.01422250316055618</v>
-      </c>
-      <c r="AC57" s="7" t="n">
-        <v>4.062091503267974</v>
-      </c>
-      <c r="AD57" s="7" t="n">
-        <v>4.026785714285714</v>
-      </c>
-      <c r="AE57" s="8" t="n">
-        <v>-0.03530578898225922</v>
-      </c>
-      <c r="AF57" s="10" t="n">
-        <v>0.9870967741935484</v>
-      </c>
-      <c r="AG57" s="10" t="n">
-        <v>0.9646017699115044</v>
-      </c>
-      <c r="AH57" s="11" t="n">
-        <v>-0.02249500428204398</v>
-      </c>
-      <c r="AI57" s="10" t="n">
-        <v>0.6852459016393443</v>
-      </c>
-      <c r="AJ57" s="10" t="n">
-        <v>0.6160714285714286</v>
-      </c>
-      <c r="AK57" s="11" t="n">
-        <v>-0.06917447306791569</v>
-      </c>
-      <c r="AL57" s="6" t="n">
-        <v>4.000000000000011</v>
-      </c>
-      <c r="AM57" s="6" t="n">
-        <v>4.000000000000006</v>
-      </c>
-      <c r="AN57" s="6" t="n">
-        <v>-4.440892098500626e-15</v>
-      </c>
-      <c r="AO57" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP57" s="10" t="n">
-        <v>0.7699115044247787</v>
-      </c>
-      <c r="AQ57" s="11" t="n">
-        <v>0.7699115044247787</v>
-      </c>
-      <c r="AR57" s="10" t="n">
-        <v>0.7419354838709677</v>
-      </c>
-      <c r="AS57" s="10" t="n">
-        <v>0.8053097345132744</v>
-      </c>
-      <c r="AT57" s="11" t="n">
-        <v>0.06337425064230662</v>
-      </c>
-      <c r="AU57" s="10" t="n">
-        <v>0.435064935064935</v>
-      </c>
-      <c r="AV57" s="10" t="n">
-        <v>0.504424778761062</v>
-      </c>
-      <c r="AW57" s="11" t="n">
-        <v>0.06935984369612691</v>
-      </c>
-      <c r="AX57" s="10" t="n">
-        <v>0.3116883116883117</v>
-      </c>
-      <c r="AY57" s="10" t="n">
-        <v>0.3008849557522124</v>
-      </c>
       <c r="AZ57" s="11" t="n">
-        <v>-0.01080335593609927</v>
+        <v>-0.2639962738705169</v>
       </c>
     </row>
     <row r="58">
@@ -11840,165 +11840,165 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>370173</v>
+        <v>12397</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>aifei(shanghai)kejiyouxiangongsi GA 30517</t>
+          <t>Ashley Furniture WI 54612</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>aifei(shanghai)kejiyouxiangongsi</t>
+          <t>Ashley Furniture</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>APS K&amp;D</t>
+          <t>Upholstery</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Eve Deng</t>
+          <t>Anne Marie Conde</t>
         </is>
       </c>
       <c r="G58" s="13" t="n">
         <v>46236</v>
       </c>
       <c r="H58" s="6" t="n">
-        <v>190</v>
+        <v>310</v>
       </c>
       <c r="I58" s="6" t="n">
         <v>113</v>
       </c>
       <c r="J58" s="6" t="n">
-        <v>-77</v>
+        <v>-197</v>
       </c>
       <c r="K58" s="7" t="n">
-        <v>2.552631578947369</v>
+        <v>1.935483870967742</v>
       </c>
       <c r="L58" s="7" t="n">
-        <v>1.849557522123894</v>
+        <v>1.265486725663717</v>
       </c>
       <c r="M58" s="8" t="n">
-        <v>-0.7030740568234748</v>
+        <v>-0.6699971453040252</v>
       </c>
       <c r="N58" s="10" t="n">
         <v>0</v>
       </c>
       <c r="O58" s="10" t="n">
-        <v>0.3628318584070797</v>
+        <v>0.504424778761062</v>
       </c>
       <c r="P58" s="11" t="n">
-        <v>0.3628318584070797</v>
+        <v>0.504424778761062</v>
       </c>
       <c r="Q58" s="7" t="n">
-        <v>4.579787234042553</v>
+        <v>3.983221476510067</v>
       </c>
       <c r="R58" s="7" t="n">
-        <v>4.433628318584071</v>
+        <v>4.086538461538462</v>
       </c>
       <c r="S58" s="8" t="n">
-        <v>-0.1461589154584821</v>
+        <v>0.1033169850283944</v>
       </c>
       <c r="T58" s="10" t="n">
-        <v>0.9368421052631579</v>
+        <v>0.8935483870967742</v>
       </c>
       <c r="U58" s="10" t="n">
-        <v>0.9823008849557522</v>
+        <v>0.8584070796460177</v>
       </c>
       <c r="V58" s="11" t="n">
-        <v>0.04545877969259426</v>
+        <v>-0.0351413074507565</v>
       </c>
       <c r="W58" s="10" t="n">
-        <v>0.9105263157894737</v>
+        <v>0.8870967741935484</v>
       </c>
       <c r="X58" s="10" t="n">
-        <v>0.9557522123893806</v>
+        <v>0.8849557522123894</v>
       </c>
       <c r="Y58" s="11" t="n">
-        <v>0.04522589659990683</v>
+        <v>-0.002141021981158953</v>
       </c>
       <c r="Z58" s="7" t="n">
-        <v>1.768421052631579</v>
+        <v>0.6071428571428571</v>
       </c>
       <c r="AA58" s="7" t="n">
-        <v>1.778761061946903</v>
+        <v>0.5929203539823009</v>
       </c>
       <c r="AB58" s="8" t="n">
-        <v>0.01034000931532386</v>
+        <v>-0.01422250316055618</v>
       </c>
       <c r="AC58" s="7" t="n">
-        <v>4.347368421052631</v>
+        <v>4.062091503267974</v>
       </c>
       <c r="AD58" s="7" t="n">
-        <v>4.141592920353983</v>
+        <v>4.026785714285714</v>
       </c>
       <c r="AE58" s="8" t="n">
-        <v>-0.2057755006986488</v>
+        <v>-0.03530578898225922</v>
       </c>
       <c r="AF58" s="10" t="n">
-        <v>0.9842105263157894</v>
+        <v>0.9870967741935484</v>
       </c>
       <c r="AG58" s="10" t="n">
-        <v>0.5929203539823009</v>
+        <v>0.9646017699115044</v>
       </c>
       <c r="AH58" s="11" t="n">
-        <v>-0.3912901723334885</v>
+        <v>-0.02249500428204398</v>
       </c>
       <c r="AI58" s="10" t="n">
-        <v>0.8631578947368421</v>
+        <v>0.6852459016393443</v>
       </c>
       <c r="AJ58" s="10" t="n">
-        <v>0.9292035398230089</v>
+        <v>0.6160714285714286</v>
       </c>
       <c r="AK58" s="11" t="n">
-        <v>0.06604564508616673</v>
+        <v>-0.06917447306791569</v>
       </c>
       <c r="AL58" s="6" t="n">
-        <v>3.000000000000009</v>
+        <v>4.000000000000011</v>
       </c>
       <c r="AM58" s="6" t="n">
-        <v>45.99999999999999</v>
+        <v>4.000000000000006</v>
       </c>
       <c r="AN58" s="6" t="n">
-        <v>42.99999999999999</v>
+        <v>-4.440892098500626e-15</v>
       </c>
       <c r="AO58" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AP58" s="10" t="n">
-        <v>0.5575221238938053</v>
+        <v>0.7699115044247787</v>
       </c>
       <c r="AQ58" s="11" t="n">
-        <v>0.5575221238938053</v>
+        <v>0.7699115044247787</v>
       </c>
       <c r="AR58" s="10" t="n">
-        <v>0.7789473684210526</v>
+        <v>0.7419354838709677</v>
       </c>
       <c r="AS58" s="10" t="n">
-        <v>0.5663716814159292</v>
+        <v>0.8053097345132744</v>
       </c>
       <c r="AT58" s="11" t="n">
-        <v>-0.2125756870051234</v>
+        <v>0.06337425064230662</v>
       </c>
       <c r="AU58" s="10" t="n">
-        <v>0.01052631578947368</v>
+        <v>0.435064935064935</v>
       </c>
       <c r="AV58" s="10" t="n">
-        <v>0.06194690265486726</v>
+        <v>0.504424778761062</v>
       </c>
       <c r="AW58" s="11" t="n">
-        <v>0.05142058686539357</v>
+        <v>0.06935984369612691</v>
       </c>
       <c r="AX58" s="10" t="n">
-        <v>0.7684210526315789</v>
+        <v>0.3116883116883117</v>
       </c>
       <c r="AY58" s="10" t="n">
-        <v>0.504424778761062</v>
+        <v>0.3008849557522124</v>
       </c>
       <c r="AZ58" s="11" t="n">
-        <v>-0.2639962738705169</v>
+        <v>-0.01080335593609927</v>
       </c>
     </row>
     <row r="59">
@@ -15200,165 +15200,165 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>322082</v>
+        <v>361472</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hangzhou Mengfeisi Home Furnishings Co., CA 92571 </t>
+          <t>Ningboyuxudianzishangwuyouxiangongsi NJ 08873</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Hangzhou Mengfeisi Home Furnishings Co., Ltd</t>
+          <t>Ningboyuxudianzishangwuyouxiangongsi</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>APS Outdoor</t>
+          <t>APS AEOF</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Moti Mao</t>
+          <t>Ricky Yu</t>
         </is>
       </c>
       <c r="G78" s="13" t="n">
         <v>46236</v>
       </c>
       <c r="H78" s="6" t="n">
-        <v>461</v>
+        <v>299</v>
       </c>
       <c r="I78" s="6" t="n">
         <v>66</v>
       </c>
       <c r="J78" s="6" t="n">
-        <v>-395</v>
+        <v>-233</v>
       </c>
       <c r="K78" s="7" t="n">
-        <v>2.414316702819957</v>
+        <v>2.468227424749164</v>
       </c>
       <c r="L78" s="7" t="n">
-        <v>1.636363636363636</v>
+        <v>1.363636363636364</v>
       </c>
       <c r="M78" s="8" t="n">
-        <v>-0.7779530664563203</v>
+        <v>-1.1045910611128</v>
       </c>
       <c r="N78" s="10" t="n">
         <v>0</v>
       </c>
       <c r="O78" s="10" t="n">
-        <v>0.3939393939393939</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="P78" s="11" t="n">
-        <v>0.3939393939393939</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="Q78" s="7" t="n">
-        <v>6.758465011286682</v>
+        <v>4.942372881355932</v>
       </c>
       <c r="R78" s="7" t="n">
-        <v>4.47457627118644</v>
+        <v>4.96969696969697</v>
       </c>
       <c r="S78" s="8" t="n">
-        <v>-2.283888740100242</v>
+        <v>0.02732408834103772</v>
       </c>
       <c r="T78" s="10" t="n">
-        <v>0.3774403470715835</v>
+        <v>0.8060200668896321</v>
       </c>
       <c r="U78" s="10" t="n">
-        <v>0.6060606060606061</v>
+        <v>0.803030303030303</v>
       </c>
       <c r="V78" s="11" t="n">
-        <v>0.2286202589890226</v>
+        <v>-0.002989763859329142</v>
       </c>
       <c r="W78" s="10" t="n">
-        <v>0.4295010845986985</v>
+        <v>0.8394648829431438</v>
       </c>
       <c r="X78" s="10" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="Y78" s="11" t="n">
-        <v>0.3886807335831198</v>
+        <v>-0.006131549609810438</v>
       </c>
       <c r="Z78" s="7" t="n">
-        <v>1.111111111111111</v>
+        <v>1.648829431438127</v>
       </c>
       <c r="AA78" s="7" t="n">
-        <v>1.333333333333333</v>
+        <v>1.242424242424242</v>
       </c>
       <c r="AB78" s="8" t="n">
-        <v>0.2222222222222221</v>
+        <v>-0.4064051890138847</v>
       </c>
       <c r="AC78" s="7" t="n">
-        <v>5.797385620915033</v>
+        <v>4.288590604026846</v>
       </c>
       <c r="AD78" s="7" t="n">
-        <v>4.46969696969697</v>
+        <v>4.075757575757576</v>
       </c>
       <c r="AE78" s="8" t="n">
-        <v>-1.327688651218063</v>
+        <v>-0.2128330282692694</v>
       </c>
       <c r="AF78" s="10" t="n">
-        <v>0.9956616052060737</v>
+        <v>0.9832775919732442</v>
       </c>
       <c r="AG78" s="10" t="n">
         <v>1</v>
       </c>
       <c r="AH78" s="11" t="n">
-        <v>0.004338394793926281</v>
+        <v>0.01672240802675584</v>
       </c>
       <c r="AI78" s="10" t="n">
-        <v>0.8300653594771242</v>
+        <v>0.8851351351351351</v>
       </c>
       <c r="AJ78" s="10" t="n">
-        <v>0.6060606060606061</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="AK78" s="11" t="n">
-        <v>-0.2240047534165182</v>
+        <v>0.02395577395577397</v>
       </c>
       <c r="AL78" s="6" t="n">
-        <v>2.000000000000016</v>
+        <v>4.999999999999996</v>
       </c>
       <c r="AM78" s="6" t="n">
         <v>0</v>
       </c>
       <c r="AN78" s="6" t="n">
-        <v>-2.000000000000016</v>
+        <v>-4.999999999999996</v>
       </c>
       <c r="AO78" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AP78" s="10" t="n">
-        <v>0.9848484848484849</v>
+        <v>1</v>
       </c>
       <c r="AQ78" s="11" t="n">
-        <v>0.9848484848484849</v>
+        <v>1</v>
       </c>
       <c r="AR78" s="10" t="n">
-        <v>0.8308026030368764</v>
+        <v>0.8294314381270903</v>
       </c>
       <c r="AS78" s="10" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.9393939393939394</v>
       </c>
       <c r="AT78" s="11" t="n">
-        <v>0.002530730296457007</v>
+        <v>0.1099625012668491</v>
       </c>
       <c r="AU78" s="10" t="n">
-        <v>0.0130718954248366</v>
+        <v>0</v>
       </c>
       <c r="AV78" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AW78" s="11" t="n">
-        <v>-0.0130718954248366</v>
+        <v>0</v>
       </c>
       <c r="AX78" s="10" t="n">
-        <v>0.8213507625272332</v>
+        <v>0.8294314381270903</v>
       </c>
       <c r="AY78" s="10" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.9393939393939394</v>
       </c>
       <c r="AZ78" s="11" t="n">
-        <v>0.01198257080610021</v>
+        <v>0.1099625012668491</v>
       </c>
     </row>
     <row r="79">
@@ -15368,165 +15368,165 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>361472</v>
+        <v>322082</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Ningboyuxudianzishangwuyouxiangongsi NJ 08873</t>
+          <t xml:space="preserve">Hangzhou Mengfeisi Home Furnishings Co., CA 92571 </t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Ningboyuxudianzishangwuyouxiangongsi</t>
+          <t>Hangzhou Mengfeisi Home Furnishings Co., Ltd</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>APS AEOF</t>
+          <t>APS Outdoor</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Ricky Yu</t>
+          <t>Moti Mao</t>
         </is>
       </c>
       <c r="G79" s="13" t="n">
         <v>46236</v>
       </c>
       <c r="H79" s="6" t="n">
-        <v>299</v>
+        <v>461</v>
       </c>
       <c r="I79" s="6" t="n">
         <v>66</v>
       </c>
       <c r="J79" s="6" t="n">
-        <v>-233</v>
+        <v>-395</v>
       </c>
       <c r="K79" s="7" t="n">
-        <v>2.468227424749164</v>
+        <v>2.414316702819957</v>
       </c>
       <c r="L79" s="7" t="n">
-        <v>1.363636363636364</v>
+        <v>1.636363636363636</v>
       </c>
       <c r="M79" s="8" t="n">
-        <v>-1.1045910611128</v>
+        <v>-0.7779530664563203</v>
       </c>
       <c r="N79" s="10" t="n">
         <v>0</v>
       </c>
       <c r="O79" s="10" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.3939393939393939</v>
       </c>
       <c r="P79" s="11" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.3939393939393939</v>
       </c>
       <c r="Q79" s="7" t="n">
-        <v>4.942372881355932</v>
+        <v>6.758465011286682</v>
       </c>
       <c r="R79" s="7" t="n">
-        <v>4.96969696969697</v>
+        <v>4.47457627118644</v>
       </c>
       <c r="S79" s="8" t="n">
-        <v>0.02732408834103772</v>
+        <v>-2.283888740100242</v>
       </c>
       <c r="T79" s="10" t="n">
-        <v>0.8060200668896321</v>
+        <v>0.3774403470715835</v>
       </c>
       <c r="U79" s="10" t="n">
-        <v>0.803030303030303</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="V79" s="11" t="n">
-        <v>-0.002989763859329142</v>
+        <v>0.2286202589890226</v>
       </c>
       <c r="W79" s="10" t="n">
-        <v>0.8394648829431438</v>
+        <v>0.4295010845986985</v>
       </c>
       <c r="X79" s="10" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8181818181818182</v>
       </c>
       <c r="Y79" s="11" t="n">
-        <v>-0.006131549609810438</v>
+        <v>0.3886807335831198</v>
       </c>
       <c r="Z79" s="7" t="n">
-        <v>1.648829431438127</v>
+        <v>1.111111111111111</v>
       </c>
       <c r="AA79" s="7" t="n">
-        <v>1.242424242424242</v>
+        <v>1.333333333333333</v>
       </c>
       <c r="AB79" s="8" t="n">
-        <v>-0.4064051890138847</v>
+        <v>0.2222222222222221</v>
       </c>
       <c r="AC79" s="7" t="n">
-        <v>4.288590604026846</v>
+        <v>5.797385620915033</v>
       </c>
       <c r="AD79" s="7" t="n">
-        <v>4.075757575757576</v>
+        <v>4.46969696969697</v>
       </c>
       <c r="AE79" s="8" t="n">
-        <v>-0.2128330282692694</v>
+        <v>-1.327688651218063</v>
       </c>
       <c r="AF79" s="10" t="n">
-        <v>0.9832775919732442</v>
+        <v>0.9956616052060737</v>
       </c>
       <c r="AG79" s="10" t="n">
         <v>1</v>
       </c>
       <c r="AH79" s="11" t="n">
-        <v>0.01672240802675584</v>
+        <v>0.004338394793926281</v>
       </c>
       <c r="AI79" s="10" t="n">
-        <v>0.8851351351351351</v>
+        <v>0.8300653594771242</v>
       </c>
       <c r="AJ79" s="10" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.6060606060606061</v>
       </c>
       <c r="AK79" s="11" t="n">
-        <v>0.02395577395577397</v>
+        <v>-0.2240047534165182</v>
       </c>
       <c r="AL79" s="6" t="n">
-        <v>4.999999999999996</v>
+        <v>2.000000000000016</v>
       </c>
       <c r="AM79" s="6" t="n">
         <v>0</v>
       </c>
       <c r="AN79" s="6" t="n">
-        <v>-4.999999999999996</v>
+        <v>-2.000000000000016</v>
       </c>
       <c r="AO79" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AP79" s="10" t="n">
-        <v>1</v>
+        <v>0.9848484848484849</v>
       </c>
       <c r="AQ79" s="11" t="n">
-        <v>1</v>
+        <v>0.9848484848484849</v>
       </c>
       <c r="AR79" s="10" t="n">
-        <v>0.8294314381270903</v>
+        <v>0.8308026030368764</v>
       </c>
       <c r="AS79" s="10" t="n">
-        <v>0.9393939393939394</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="AT79" s="11" t="n">
-        <v>0.1099625012668491</v>
+        <v>0.002530730296457007</v>
       </c>
       <c r="AU79" s="10" t="n">
-        <v>0</v>
+        <v>0.0130718954248366</v>
       </c>
       <c r="AV79" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AW79" s="11" t="n">
-        <v>0</v>
+        <v>-0.0130718954248366</v>
       </c>
       <c r="AX79" s="10" t="n">
-        <v>0.8294314381270903</v>
+        <v>0.8213507625272332</v>
       </c>
       <c r="AY79" s="10" t="n">
-        <v>0.9393939393939394</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="AZ79" s="11" t="n">
-        <v>0.1099625012668491</v>
+        <v>0.01198257080610021</v>
       </c>
     </row>
     <row r="80">
@@ -16775,12 +16775,12 @@
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="23" customWidth="1" min="23" max="23"/>
-    <col width="24" customWidth="1" min="24" max="24"/>
-    <col width="25" customWidth="1" min="25" max="25"/>
+    <col width="33" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="21" max="21"/>
+    <col width="31" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="21" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
     <col width="16" customWidth="1" min="26" max="26"/>
     <col width="17" customWidth="1" min="27" max="27"/>
     <col width="18" customWidth="1" min="28" max="28"/>
@@ -16908,32 +16908,32 @@
       </c>
       <c r="T1" s="12" t="inlineStr">
         <is>
-          <t>pre_fast_badge</t>
+          <t>Pre Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="U1" s="12" t="inlineStr">
         <is>
-          <t>post_fast_badge</t>
+          <t>Post Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="V1" s="12" t="inlineStr">
         <is>
-          <t>delta_fast_badge</t>
+          <t>Δ Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="W1" s="12" t="inlineStr">
         <is>
-          <t>pre_actual_fast_badge</t>
+          <t>Pre actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="X1" s="12" t="inlineStr">
         <is>
-          <t>post_actual_fast_badge</t>
+          <t>Post actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="Y1" s="12" t="inlineStr">
         <is>
-          <t>delta_actual_fast_badge</t>
+          <t>Δ actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="Z1" s="12" t="inlineStr">
@@ -31542,12 +31542,12 @@
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="23" customWidth="1" min="23" max="23"/>
-    <col width="24" customWidth="1" min="24" max="24"/>
-    <col width="25" customWidth="1" min="25" max="25"/>
+    <col width="33" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="21" max="21"/>
+    <col width="31" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="21" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
     <col width="16" customWidth="1" min="26" max="26"/>
     <col width="17" customWidth="1" min="27" max="27"/>
     <col width="18" customWidth="1" min="28" max="28"/>
@@ -31675,32 +31675,32 @@
       </c>
       <c r="T1" s="12" t="inlineStr">
         <is>
-          <t>pre_fast_badge</t>
+          <t>Pre Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="U1" s="12" t="inlineStr">
         <is>
-          <t>post_fast_badge</t>
+          <t>Post Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="V1" s="12" t="inlineStr">
         <is>
-          <t>delta_fast_badge</t>
+          <t>Δ Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="W1" s="12" t="inlineStr">
         <is>
-          <t>pre_actual_fast_badge</t>
+          <t>Pre actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="X1" s="12" t="inlineStr">
         <is>
-          <t>post_actual_fast_badge</t>
+          <t>Post actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="Y1" s="12" t="inlineStr">
         <is>
-          <t>delta_actual_fast_badge</t>
+          <t>Δ actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="Z1" s="12" t="inlineStr">
@@ -42262,165 +42262,165 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>153347</v>
+        <v>347934</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Alphamarts TX 77521(2)</t>
+          <t>Ningbo Jiangbei Fufu CA 91761 (3)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Alphamarts</t>
+          <t>Ningbo Jiangbei Fufu</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>APS Outdoor</t>
+          <t>APS Bedroom</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Melody Lu</t>
+          <t>Christal Ding</t>
         </is>
       </c>
       <c r="G64" s="13" t="n">
         <v>46236</v>
       </c>
       <c r="H64" s="6" t="n">
-        <v>842</v>
+        <v>495</v>
       </c>
       <c r="I64" s="6" t="n">
         <v>191</v>
       </c>
       <c r="J64" s="6" t="n">
-        <v>-651</v>
+        <v>-304</v>
       </c>
       <c r="K64" s="7" t="n">
-        <v>1.235154394299287</v>
+        <v>1.395959595959596</v>
       </c>
       <c r="L64" s="7" t="n">
-        <v>1.036649214659686</v>
+        <v>1.073298429319372</v>
       </c>
       <c r="M64" s="8" t="n">
-        <v>-0.1985051796396013</v>
+        <v>-0.3226611666402244</v>
       </c>
       <c r="N64" s="10" t="n">
-        <v>0.9002375296912114</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="O64" s="10" t="n">
         <v>0.9633507853403142</v>
       </c>
       <c r="P64" s="11" t="n">
-        <v>0.06311325564910275</v>
+        <v>0.09668411867364746</v>
       </c>
       <c r="Q64" s="7" t="n">
-        <v>4.059259259259259</v>
+        <v>5.377358490566038</v>
       </c>
       <c r="R64" s="7" t="n">
-        <v>3.360215053763441</v>
+        <v>4.648351648351649</v>
       </c>
       <c r="S64" s="8" t="n">
-        <v>-0.6990442054958184</v>
+        <v>-0.7290068422143889</v>
       </c>
       <c r="T64" s="10" t="n">
-        <v>0.8657957244655582</v>
+        <v>0.6404040404040404</v>
       </c>
       <c r="U64" s="10" t="n">
-        <v>0.9476439790575916</v>
+        <v>0.7277486910994765</v>
       </c>
       <c r="V64" s="11" t="n">
-        <v>0.08184825459203338</v>
+        <v>0.08734465069543607</v>
       </c>
       <c r="W64" s="10" t="n">
-        <v>0.8966745843230404</v>
+        <v>0.6383838383838384</v>
       </c>
       <c r="X64" s="10" t="n">
+        <v>0.7643979057591623</v>
+      </c>
+      <c r="Y64" s="11" t="n">
+        <v>0.1260140673753239</v>
+      </c>
+      <c r="Z64" s="7" t="n">
+        <v>1.167676767676768</v>
+      </c>
+      <c r="AA64" s="7" t="n">
+        <v>0.9738219895287958</v>
+      </c>
+      <c r="AB64" s="8" t="n">
+        <v>-0.1938547781479718</v>
+      </c>
+      <c r="AC64" s="7" t="n">
+        <v>5.016194331983805</v>
+      </c>
+      <c r="AD64" s="7" t="n">
+        <v>4.240837696335078</v>
+      </c>
+      <c r="AE64" s="8" t="n">
+        <v>-0.7753566356487269</v>
+      </c>
+      <c r="AF64" s="10" t="n">
+        <v>0.7818181818181819</v>
+      </c>
+      <c r="AG64" s="10" t="n">
         <v>0.9528795811518325</v>
       </c>
-      <c r="Y64" s="11" t="n">
-        <v>0.0562049968287921</v>
-      </c>
-      <c r="Z64" s="7" t="n">
-        <v>1.103571428571429</v>
-      </c>
-      <c r="AA64" s="7" t="n">
-        <v>0.7958115183246073</v>
-      </c>
-      <c r="AB64" s="8" t="n">
-        <v>-0.3077599102468214</v>
-      </c>
-      <c r="AC64" s="7" t="n">
-        <v>3.65554231227652</v>
-      </c>
-      <c r="AD64" s="7" t="n">
-        <v>2.936842105263158</v>
-      </c>
-      <c r="AE64" s="8" t="n">
-        <v>-0.7187002070133621</v>
-      </c>
-      <c r="AF64" s="10" t="n">
-        <v>0.8764845605700713</v>
-      </c>
-      <c r="AG64" s="10" t="n">
-        <v>0.9842931937172775</v>
-      </c>
       <c r="AH64" s="11" t="n">
-        <v>0.1078086331472062</v>
+        <v>0.1710613993336506</v>
       </c>
       <c r="AI64" s="10" t="n">
-        <v>0.815035799522673</v>
+        <v>0.7221095334685599</v>
       </c>
       <c r="AJ64" s="10" t="n">
-        <v>0.8263157894736842</v>
+        <v>0.806282722513089</v>
       </c>
       <c r="AK64" s="11" t="n">
-        <v>0.0112799899510112</v>
+        <v>0.08417318904452908</v>
       </c>
       <c r="AL64" s="6" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="AM64" s="6" t="n">
-        <v>2.999999999999992</v>
+        <v>8.999999999999998</v>
       </c>
       <c r="AN64" s="6" t="n">
-        <v>-101</v>
+        <v>-98.99999999999999</v>
       </c>
       <c r="AO64" s="10" t="n">
-        <v>0</v>
+        <v>0.00404040404040404</v>
       </c>
       <c r="AP64" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AQ64" s="11" t="n">
-        <v>0</v>
+        <v>-0.00404040404040404</v>
       </c>
       <c r="AR64" s="10" t="n">
-        <v>0.01900237529691211</v>
+        <v>0.01414141414141414</v>
       </c>
       <c r="AS64" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AT64" s="11" t="n">
-        <v>-0.01900237529691211</v>
+        <v>-0.01414141414141414</v>
       </c>
       <c r="AU64" s="10" t="n">
-        <v>0.01071428571428571</v>
+        <v>0.01414141414141414</v>
       </c>
       <c r="AV64" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AW64" s="11" t="n">
-        <v>-0.01071428571428571</v>
+        <v>-0.01414141414141414</v>
       </c>
       <c r="AX64" s="10" t="n">
-        <v>0.008333333333333333</v>
+        <v>0</v>
       </c>
       <c r="AY64" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AZ64" s="11" t="n">
-        <v>-0.008333333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -42430,165 +42430,165 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>347934</v>
+        <v>153347</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Ningbo Jiangbei Fufu CA 91761 (3)</t>
+          <t>Alphamarts TX 77521(2)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Ningbo Jiangbei Fufu</t>
+          <t>Alphamarts</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>APS Bedroom</t>
+          <t>APS Outdoor</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Christal Ding</t>
+          <t>Melody Lu</t>
         </is>
       </c>
       <c r="G65" s="13" t="n">
         <v>46236</v>
       </c>
       <c r="H65" s="6" t="n">
-        <v>495</v>
+        <v>842</v>
       </c>
       <c r="I65" s="6" t="n">
         <v>191</v>
       </c>
       <c r="J65" s="6" t="n">
-        <v>-304</v>
+        <v>-651</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>1.395959595959596</v>
+        <v>1.235154394299287</v>
       </c>
       <c r="L65" s="7" t="n">
-        <v>1.073298429319372</v>
+        <v>1.036649214659686</v>
       </c>
       <c r="M65" s="8" t="n">
-        <v>-0.3226611666402244</v>
+        <v>-0.1985051796396013</v>
       </c>
       <c r="N65" s="10" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.9002375296912114</v>
       </c>
       <c r="O65" s="10" t="n">
         <v>0.9633507853403142</v>
       </c>
       <c r="P65" s="11" t="n">
-        <v>0.09668411867364746</v>
+        <v>0.06311325564910275</v>
       </c>
       <c r="Q65" s="7" t="n">
-        <v>5.377358490566038</v>
+        <v>4.059259259259259</v>
       </c>
       <c r="R65" s="7" t="n">
-        <v>4.648351648351649</v>
+        <v>3.360215053763441</v>
       </c>
       <c r="S65" s="8" t="n">
-        <v>-0.7290068422143889</v>
+        <v>-0.6990442054958184</v>
       </c>
       <c r="T65" s="10" t="n">
-        <v>0.6404040404040404</v>
+        <v>0.8657957244655582</v>
       </c>
       <c r="U65" s="10" t="n">
-        <v>0.7277486910994765</v>
+        <v>0.9476439790575916</v>
       </c>
       <c r="V65" s="11" t="n">
-        <v>0.08734465069543607</v>
+        <v>0.08184825459203338</v>
       </c>
       <c r="W65" s="10" t="n">
-        <v>0.6383838383838384</v>
+        <v>0.8966745843230404</v>
       </c>
       <c r="X65" s="10" t="n">
-        <v>0.7643979057591623</v>
+        <v>0.9528795811518325</v>
       </c>
       <c r="Y65" s="11" t="n">
-        <v>0.1260140673753239</v>
+        <v>0.0562049968287921</v>
       </c>
       <c r="Z65" s="7" t="n">
-        <v>1.167676767676768</v>
+        <v>1.103571428571429</v>
       </c>
       <c r="AA65" s="7" t="n">
-        <v>0.9738219895287958</v>
+        <v>0.7958115183246073</v>
       </c>
       <c r="AB65" s="8" t="n">
-        <v>-0.1938547781479718</v>
+        <v>-0.3077599102468214</v>
       </c>
       <c r="AC65" s="7" t="n">
-        <v>5.016194331983805</v>
+        <v>3.65554231227652</v>
       </c>
       <c r="AD65" s="7" t="n">
-        <v>4.240837696335078</v>
+        <v>2.936842105263158</v>
       </c>
       <c r="AE65" s="8" t="n">
-        <v>-0.7753566356487269</v>
+        <v>-0.7187002070133621</v>
       </c>
       <c r="AF65" s="10" t="n">
-        <v>0.7818181818181819</v>
+        <v>0.8764845605700713</v>
       </c>
       <c r="AG65" s="10" t="n">
-        <v>0.9528795811518325</v>
+        <v>0.9842931937172775</v>
       </c>
       <c r="AH65" s="11" t="n">
-        <v>0.1710613993336506</v>
+        <v>0.1078086331472062</v>
       </c>
       <c r="AI65" s="10" t="n">
-        <v>0.7221095334685599</v>
+        <v>0.815035799522673</v>
       </c>
       <c r="AJ65" s="10" t="n">
-        <v>0.806282722513089</v>
+        <v>0.8263157894736842</v>
       </c>
       <c r="AK65" s="11" t="n">
-        <v>0.08417318904452908</v>
+        <v>0.0112799899510112</v>
       </c>
       <c r="AL65" s="6" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="AM65" s="6" t="n">
-        <v>8.999999999999998</v>
+        <v>2.999999999999992</v>
       </c>
       <c r="AN65" s="6" t="n">
-        <v>-98.99999999999999</v>
+        <v>-101</v>
       </c>
       <c r="AO65" s="10" t="n">
-        <v>0.00404040404040404</v>
+        <v>0</v>
       </c>
       <c r="AP65" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AQ65" s="11" t="n">
-        <v>-0.00404040404040404</v>
+        <v>0</v>
       </c>
       <c r="AR65" s="10" t="n">
-        <v>0.01414141414141414</v>
+        <v>0.01900237529691211</v>
       </c>
       <c r="AS65" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AT65" s="11" t="n">
-        <v>-0.01414141414141414</v>
+        <v>-0.01900237529691211</v>
       </c>
       <c r="AU65" s="10" t="n">
-        <v>0.01414141414141414</v>
+        <v>0.01071428571428571</v>
       </c>
       <c r="AV65" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AW65" s="11" t="n">
-        <v>-0.01414141414141414</v>
+        <v>-0.01071428571428571</v>
       </c>
       <c r="AX65" s="10" t="n">
-        <v>0</v>
+        <v>0.008333333333333333</v>
       </c>
       <c r="AY65" s="10" t="n">
         <v>0</v>
       </c>
       <c r="AZ65" s="11" t="n">
-        <v>0</v>
+        <v>-0.008333333333333333</v>
       </c>
     </row>
     <row r="66">
@@ -46189,12 +46189,12 @@
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="23" customWidth="1" min="23" max="23"/>
-    <col width="24" customWidth="1" min="24" max="24"/>
-    <col width="25" customWidth="1" min="25" max="25"/>
+    <col width="33" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="21" max="21"/>
+    <col width="31" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="21" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
     <col width="16" customWidth="1" min="26" max="26"/>
     <col width="17" customWidth="1" min="27" max="27"/>
     <col width="18" customWidth="1" min="28" max="28"/>
@@ -46322,32 +46322,32 @@
       </c>
       <c r="T1" s="12" t="inlineStr">
         <is>
-          <t>pre_fast_badge</t>
+          <t>Pre Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="U1" s="12" t="inlineStr">
         <is>
-          <t>post_fast_badge</t>
+          <t>Post Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="V1" s="12" t="inlineStr">
         <is>
-          <t>delta_fast_badge</t>
+          <t>Δ Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="W1" s="12" t="inlineStr">
         <is>
-          <t>pre_actual_fast_badge</t>
+          <t>Pre actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="X1" s="12" t="inlineStr">
         <is>
-          <t>post_actual_fast_badge</t>
+          <t>Post actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="Y1" s="12" t="inlineStr">
         <is>
-          <t>delta_actual_fast_badge</t>
+          <t>Δ actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="Z1" s="12" t="inlineStr">
@@ -52338,8 +52338,8 @@
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="19" customWidth="1" min="18" max="18"/>
+    <col width="29" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="15" customWidth="1" min="20" max="20"/>
   </cols>
@@ -52427,12 +52427,12 @@
       </c>
       <c r="Q1" s="12" t="inlineStr">
         <is>
-          <t>fast_badge</t>
+          <t>Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="R1" s="12" t="inlineStr">
         <is>
-          <t>actual_fast_badge</t>
+          <t>Actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="S1" s="12" t="inlineStr">
@@ -54107,8 +54107,8 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="29" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
@@ -54185,12 +54185,12 @@
       </c>
       <c r="O1" s="12" t="inlineStr">
         <is>
-          <t>fast_badge</t>
+          <t>Fast badge (stated O2D ≤ 5)</t>
         </is>
       </c>
       <c r="P1" s="12" t="inlineStr">
         <is>
-          <t>actual_fast_badge</t>
+          <t>Actual O2D ≤ 5</t>
         </is>
       </c>
       <c r="Q1" s="12" t="inlineStr">

</xml_diff>